<commit_message>
refactor changes and noramlization
</commit_message>
<xml_diff>
--- a/data/output/evaluation/openai/internal-consistency/all-criteria/rank_comparison.xlsx
+++ b/data/output/evaluation/openai/internal-consistency/all-criteria/rank_comparison.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,10 +447,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C2" t="n">
-        <v>9.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -460,10 +460,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="C3" t="n">
-        <v>5.4</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="4">
@@ -473,10 +473,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="C4" t="n">
-        <v>7.4</v>
+        <v>8.714285714285714</v>
       </c>
     </row>
     <row r="5">
@@ -486,10 +486,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>8.666666666666666</v>
       </c>
       <c r="C5" t="n">
-        <v>8.25</v>
+        <v>8.666666666666666</v>
       </c>
     </row>
     <row r="6">
@@ -499,218 +499,179 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>8</v>
+        <v>8.166666666666666</v>
       </c>
       <c r="C6" t="n">
-        <v>9.25</v>
+        <v>8.428571428571429</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Komoot</t>
+          <t>Map My Run</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>3.3</v>
       </c>
       <c r="C7" t="n">
-        <v>8</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Map My Run</t>
+          <t>MyFitnessPal</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>4.1</v>
+        <v>6.777777777777778</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>MyFitnessPal</t>
+          <t>Nike Run Club</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C9" t="n">
-        <v>5.25</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Nike Run Club</t>
+          <t>Pacer Pedometer</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>7.625</v>
       </c>
       <c r="C10" t="n">
-        <v>2.1</v>
+        <v>7.25</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Pacer</t>
+          <t>Pumatrac</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>Pacer Pedometer &amp; Step Tracker</t>
+          <t>Runkeeper</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7</v>
+        <v>4.9</v>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Polar Flow</t>
+          <t>Runtastic</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0</v>
+        <v>5.8</v>
       </c>
       <c r="C13" t="n">
-        <v>9</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>Pumatrac</t>
+          <t>Samsung Health</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0</v>
+        <v>9.666666666666666</v>
       </c>
       <c r="C14" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>Runkeeper</t>
+          <t>Sports Tracker</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4.4</v>
+        <v>9</v>
       </c>
       <c r="C15" t="n">
-        <v>4.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>Runtastic</t>
+          <t>Strava</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5.8</v>
+        <v>1</v>
       </c>
       <c r="C16" t="n">
-        <v>5.9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>Samsung Health</t>
+          <t>Under Armour Record</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C17" t="n">
-        <v>9</v>
+        <v>8.666666666666666</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>Sports Tracker</t>
+          <t>Zombies, Run!</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="C18" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>Strava</t>
+          <t>Zwift</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C19" t="n">
-        <v>1.1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>Under Armour Record</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>0</v>
-      </c>
-      <c r="C20" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>Zombies, Run!</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>0</v>
-      </c>
-      <c r="C21" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>Zwift</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>0</v>
-      </c>
-      <c r="C22" t="n">
-        <v>9</v>
+        <v>8.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>